<commit_message>
no puedo sincronizar este reporte
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Repositorios de capturas y reportes\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DEBEC3-352C-41C2-BEFC-2CA867FA63E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FB5703-AA99-4E1D-BFD4-A7571F14A325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="181">
   <si>
     <t>Fecha</t>
   </si>
@@ -243,9 +243,6 @@
     <t>El Sol de Hidalgo</t>
   </si>
   <si>
-    <t>La Jornada Hidalgo</t>
-  </si>
-  <si>
     <t>OCSAD</t>
   </si>
   <si>
@@ -288,15 +285,9 @@
     <t>Pachuca Brilla</t>
   </si>
   <si>
-    <t>Homicidio de sacerdote</t>
-  </si>
-  <si>
     <t>Tarifario de taxis</t>
   </si>
   <si>
-    <t>Ataque Armado</t>
-  </si>
-  <si>
     <t>OEEH</t>
   </si>
   <si>
@@ -306,292 +297,289 @@
     <t>Cintillo</t>
   </si>
   <si>
-    <t>Gimnasiada Nacional</t>
-  </si>
-  <si>
     <t>Plaza Juárez</t>
   </si>
   <si>
-    <t>Accidente transporte público</t>
-  </si>
-  <si>
-    <t>Temas internacionales</t>
-  </si>
-  <si>
-    <t>Bloquean para exigir obras... serán escuchados</t>
-  </si>
-  <si>
-    <t>Bloqueo Carretero</t>
-  </si>
-  <si>
-    <t>Incrementan 20.4 % fraudes en la entidad</t>
-  </si>
-  <si>
-    <t>Fraude</t>
-  </si>
-  <si>
-    <t>Teléfonos celulares, ni en clases ni en el recreo</t>
-  </si>
-  <si>
     <t>Regulación de dispositivos digitales</t>
   </si>
   <si>
-    <t>Subirán 20% tarifas del servicio de taxi: usuarios consideran elevado el nuevo costo y piden que entre el serviio de plataformas</t>
-  </si>
-  <si>
-    <t>Proveedores quedaron a deber medicamento</t>
-  </si>
-  <si>
-    <t>Salud</t>
-  </si>
-  <si>
-    <t>Abasto De Medicamentos</t>
-  </si>
-  <si>
-    <t>Celulares en escuelas, solo para emergencias</t>
-  </si>
-  <si>
-    <t>Prevén más de 10 mil candidaturas en 2027</t>
-  </si>
-  <si>
-    <t>Elecciones</t>
-  </si>
-  <si>
-    <t>Aumenta tarifa de taxis en Pachuca y La Reforma</t>
-  </si>
-  <si>
-    <t>Bloquean 6 horas la Pachuca-Sahagún</t>
-  </si>
-  <si>
-    <t>Cierre Carretero</t>
-  </si>
-  <si>
-    <t>Siguen 3 pistas en caso párroco</t>
-  </si>
-  <si>
-    <t>Xotec: fusiona lucha libre y teatro en el cuadrilátero</t>
-  </si>
-  <si>
-    <t>Evento Cultural</t>
-  </si>
-  <si>
-    <t>Tocan fondo</t>
-  </si>
-  <si>
-    <t>Clasifican a gimnasiada</t>
-  </si>
-  <si>
     <t>Inhide</t>
   </si>
   <si>
-    <t>Acumulan más accidentes las Rutas 47 y 108</t>
-  </si>
-  <si>
-    <t>STCH</t>
-  </si>
-  <si>
-    <t>Van 2 carpetas de investigación por tentativa de feminicidio</t>
-  </si>
-  <si>
-    <t>Feminicidio</t>
-  </si>
-  <si>
-    <t>Presentan nueva tarifa de taxis</t>
-  </si>
-  <si>
-    <t>Asael llama a sus homólogos a cerrar filas por el presupuesto</t>
-  </si>
-  <si>
-    <t>Modificación Presupuestal</t>
-  </si>
-  <si>
-    <t>Pachuca plantea ley de ingresos por 1,603 mdp</t>
-  </si>
-  <si>
-    <t>Ley De Ingresos</t>
-  </si>
-  <si>
-    <t>Servicio de taxis aumenta tarifa, pondrán límite con dispositivos</t>
-  </si>
-  <si>
-    <t>Inteligencia artificial: hora de actuar</t>
-  </si>
-  <si>
-    <t>Inteligencia Artificial</t>
-  </si>
-  <si>
-    <t>Debate sobre IA y celulares en los 475 años de la Universidad</t>
-  </si>
-  <si>
-    <t>La Diócesis de Huejutla colabora en investigación</t>
-  </si>
-  <si>
-    <t>Ataques de Estados Unidos a lanchas son ""Ejecuciones extrajudiciales"": ONU</t>
-  </si>
-  <si>
-    <t>El retiro de celulares debe ser con acuerdos, pide Natividad Castrejón</t>
-  </si>
-  <si>
-    <t>Caen tres tras balacera</t>
-  </si>
-  <si>
-    <t>Tarifa de taxis incrementará 20%: Semot</t>
-  </si>
-  <si>
-    <t>Acuerdan prohibir uso de celulares en primaria y secundaria</t>
-  </si>
-  <si>
-    <t>El titular de la SEPH, Natividad Castrejón Valdez, precisó que no se trata de una prohibición, sino de una restricción. Explicó que en nivel  básico no podrán utilizarse celulares o tabletas, salvo en actividades académicas; en secundaria podrán emplearse en casos de emergencia,  pero deberán permanecer apagados durante toda la jornada escolar.</t>
-  </si>
-  <si>
-    <t>Fotonota</t>
-  </si>
-  <si>
-    <t>Violencia deja 9 muertos en Morelos y Guanajuato</t>
-  </si>
-  <si>
-    <t>Ola De Violencia</t>
-  </si>
-  <si>
-    <t>Una cosa es perder terreno en infraestructura o mercado laboral, temas que se corrigen con obra pública y política de empleo, y otra muy distinta es retroceder en derecho o en sistema político y gobiernos, donde el deterioro habla de percepción de seguridad, corrupción o manejo de finanzas públicas”.</t>
-  </si>
-  <si>
-    <t>Informe De Gobierno</t>
-  </si>
-  <si>
-    <t>Anuncian aumento del 20% en la tarifa de taxis; ajuste iniciará en Pachuca y La Reforma</t>
-  </si>
-  <si>
-    <t>Uso de celulares en escuelas  solo para emergencias o  actividades planeadas: SEPH</t>
-  </si>
-  <si>
-    <t>Exigen reparación integral tras muerte de  Karla y lesiones de Estrella</t>
-  </si>
-  <si>
-    <t>Atropellamiento estudiante</t>
-  </si>
-  <si>
-    <t>Siguen tres líneas de investigación por muerte de párroco de Huejutla</t>
-  </si>
-  <si>
-    <t>Participarán 139 artesanos en la Feria San Francisco Hidalgo 2026</t>
-  </si>
-  <si>
-    <t>Taxis en Hidalgo aumentarán 20% su tarifa</t>
-  </si>
-  <si>
-    <t>Hidalgo, entre estados con mayor crecimiento del PIB y avance en empleo: IMCO</t>
-  </si>
-  <si>
     <t>Crecimiento Económico</t>
   </si>
   <si>
-    <t>Interceptan a pareja que transportaba 72 kilos de marihuana</t>
-  </si>
-  <si>
-    <t>Combate Al Narcomenudeo</t>
-  </si>
-  <si>
-    <t>Piden 25 millones de reparación por muerte de Karla</t>
-  </si>
-  <si>
-    <t>¡Adiós celulares!</t>
-  </si>
-  <si>
-    <t>Tuzobús ampliará servicio durante la Feria</t>
-  </si>
-  <si>
-    <t>Sitmah</t>
-  </si>
-  <si>
-    <t>Regularán uso de celulares en escuelas de Hidalgo</t>
-  </si>
-  <si>
-    <t>Sube 20% tarifa de taxis en Pachuca y Mineral de la Reforma</t>
-  </si>
-  <si>
-    <t>En operativo coordinado por el Gabinete de Seguridad, detienen a tres personas tras altercado en Pachuca</t>
-  </si>
-  <si>
-    <t>Reunión Gabinete De Seguridad</t>
-  </si>
-  <si>
-    <t>Ana María Rivera inaugura red eléctrica en Tezontepec de Aldama</t>
-  </si>
-  <si>
-    <t>Obras De Infraestructura</t>
-  </si>
-  <si>
-    <t>Entrega Claudia Sandoval mobiliario a Primaria de Tlamaco</t>
-  </si>
-  <si>
-    <t>Entrega De Equipo Escolar</t>
-  </si>
-  <si>
-    <t>Said Vargas continúa con el acercamiento a la base magisterial</t>
-  </si>
-  <si>
     <t>Reunión con sindicato</t>
   </si>
   <si>
-    <t>Trabajo en equipo entre DIFH y DIF Huejutla amplía apoyos para grupos prioritarios</t>
-  </si>
-  <si>
-    <t>Cobertura de apoyos sociales</t>
-  </si>
-  <si>
-    <t>Garza Leal</t>
-  </si>
-  <si>
-    <t>Publicidad comercial</t>
-  </si>
-  <si>
-    <t>Actualizan tarifa de taxis en Hidalgo; buscan fortalecer calidad del servicio</t>
-  </si>
-  <si>
-    <t>Todo listo para la edición 2026 de la Feria de San Francisco</t>
-  </si>
-  <si>
-    <t>Carlos Rivera pone pausa a su carrera tras concierto en el Grito</t>
-  </si>
-  <si>
-    <t>Grito De Independencia</t>
-  </si>
-  <si>
-    <t>Educación integral: el estado evalúa aprendizajes, cuida emociones y promueve tecnología responsable</t>
-  </si>
-  <si>
-    <t>Fortalecimiento educativo</t>
-  </si>
-  <si>
-    <t>Gabinete de Seguridad detiene a tres personas tras altercado en Pachuca</t>
-  </si>
-  <si>
-    <t>Un espacio para encontrarnos</t>
-  </si>
-  <si>
-    <t>Apoyo a artesanos</t>
-  </si>
-  <si>
     <t>Con la pirotecnia no se juega</t>
   </si>
   <si>
     <t>Pirotecnia</t>
   </si>
   <si>
-    <t>Tarifa mínima de taxis aumentará a 45 pesos</t>
-  </si>
-  <si>
-    <t>Capturan a pareja con 72 kilos de presunta marihuana</t>
-  </si>
-  <si>
-    <t>Restringen uso de dispositivos móviles en aulas</t>
-  </si>
-  <si>
-    <t>Audiencia por triple feminicidio, continuará el jueves</t>
-  </si>
-  <si>
-    <t>Proceso Por Feminicidio</t>
+    <t>Crece vivienda más que población: Inegi</t>
+  </si>
+  <si>
+    <t>Dinámica demográfica</t>
+  </si>
+  <si>
+    <t>Aún sin llegar la maquinaria</t>
+  </si>
+  <si>
+    <t>Conagua</t>
+  </si>
+  <si>
+    <t>Control lirio acuático</t>
+  </si>
+  <si>
+    <t>Piden que maestros tampoco usen celular</t>
+  </si>
+  <si>
+    <t>Mendoza llama a revisar estrategia de seguridad</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Intervención extranjera</t>
+  </si>
+  <si>
+    <t>Rinden homenaje a Juana Alarcón</t>
+  </si>
+  <si>
+    <t>Deceso de diputada</t>
+  </si>
+  <si>
+    <t>Registra Inegi 19 mil desplazamientos por desastres y violencia</t>
+  </si>
+  <si>
+    <t>Taxis en Pachuca, deteriorados</t>
+  </si>
+  <si>
+    <t>Viajan con sabor huasteco</t>
+  </si>
+  <si>
+    <t>Temas varios</t>
+  </si>
+  <si>
+    <t>En Tizayuca, transporte público provoca accidentes</t>
+  </si>
+  <si>
+    <t>Deficiencias transporte público</t>
+  </si>
+  <si>
+    <t>Pausan llamado de leigisladora suplente</t>
+  </si>
+  <si>
+    <t>Diputado suplente</t>
+  </si>
+  <si>
+    <t>Celebran a universidades tecnológicas y politécnicas</t>
+  </si>
+  <si>
+    <t>Conmemoración Aniversario</t>
+  </si>
+  <si>
+    <t>Pendiente, homologar sueldo a nivel federal en Tecnológicos</t>
+  </si>
+  <si>
+    <t>Universidades</t>
+  </si>
+  <si>
+    <t>Homologación salarial</t>
+  </si>
+  <si>
+    <t>Ve gobernador libertad en las manifestaciones en los informes</t>
+  </si>
+  <si>
+    <t>Manifestación informe</t>
+  </si>
+  <si>
+    <t>Vigilaría Congreso el servicio de transporte</t>
+  </si>
+  <si>
+    <t>Cesaron al Rambo</t>
+  </si>
+  <si>
+    <t>Dan el último adiós a la dip. Juana Alarcón</t>
+  </si>
+  <si>
+    <t>Realiza DIFH entrega de 305 becas pilaress</t>
+  </si>
+  <si>
+    <t>Pilares</t>
+  </si>
+  <si>
+    <t>IMCO: Hidalgo registra avances en economía, salud y seguridad</t>
+  </si>
+  <si>
+    <t>Desplazamientos y dependencia de apoyos revela encuesta del Inegi</t>
+  </si>
+  <si>
+    <t>Celebran a las universidades tecnológicas y politécnicas</t>
+  </si>
+  <si>
+    <t>Brecha laboral: Participación masculina es de 6 por cada 4 mujeres</t>
+  </si>
+  <si>
+    <t>Brecha de género</t>
+  </si>
+  <si>
+    <t>Trump compara a los cárteles de México co el grupo ISIS</t>
+  </si>
+  <si>
+    <t>Traerán debate sobre futuro e innovación</t>
+  </si>
+  <si>
+    <t>Abren la posibilidad para demandar a plataformas digitales en nuestro país</t>
+  </si>
+  <si>
+    <t>Next Energy pide se revise el caso de su propietario preso</t>
+  </si>
+  <si>
+    <t>Viajan en vehículo articular apenas 1.5 personas</t>
+  </si>
+  <si>
+    <t>Movilidad urbana</t>
+  </si>
+  <si>
+    <t>Aumenta 14.9 puntos porcentuales la eficiencia terminal en universidades de la entidad</t>
+  </si>
+  <si>
+    <t>Eficiencia terminal</t>
+  </si>
+  <si>
+    <t>Hidalgo suma 162 mil habitantes y alcanza una población de 3.2 millones</t>
+  </si>
+  <si>
+    <t>Menchaca pide a su gabinete prepararse para comparecencias ante el Congreso</t>
+  </si>
+  <si>
+    <t>Comparecencias</t>
+  </si>
+  <si>
+    <t>Rinden homenaje póstumo a la diputada Juana Olivia Alarcón</t>
+  </si>
+  <si>
+    <t>Pachuca tendrá ingreso de 1.6 mdp por espectáculos de la Feria San Francisco</t>
+  </si>
+  <si>
+    <t>Sin firma, no hay pruebas contra Osorio Chong por desvío en Policía Federal: Secretaría Anticorrupción</t>
+  </si>
+  <si>
+    <t>Corrupción</t>
+  </si>
+  <si>
+    <t>Uber y DIDI siguen prohibidos en Hidalgo</t>
+  </si>
+  <si>
+    <t>Apps de transporte</t>
+  </si>
+  <si>
+    <t>DIFH entrega becas a 305 niños de 17 municipios</t>
+  </si>
+  <si>
+    <t>Hidalgo, sede de la Olimpiada Nacional 2027</t>
+  </si>
+  <si>
+    <t>Olimpiada Nacional</t>
+  </si>
+  <si>
+    <t>Aumentan a 84.5% los estudiantes que logran concluir universidad</t>
+  </si>
+  <si>
+    <t>Hidalgo ya supera los 3.2 millones de habitantes</t>
+  </si>
+  <si>
+    <t>Hidalgo buscará regresar al top 15 en competitividad</t>
+  </si>
+  <si>
+    <t>La tarifa sube, ¿y el servicio?</t>
+  </si>
+  <si>
+    <t>Editorial</t>
+  </si>
+  <si>
+    <t>Invita Semot a fomentar el respeto a la jerarquía de la movilidad</t>
+  </si>
+  <si>
+    <t>Jerarquía de la Movilidad</t>
+  </si>
+  <si>
+    <t>Tula fortalece su capacidad operativa en seguridad con inversión superior a 6 mdp</t>
+  </si>
+  <si>
+    <t>Fortalecimiento Policiaco</t>
+  </si>
+  <si>
+    <t>Obras tienen un año de garantía por vicios ocultos: Sipdus</t>
+  </si>
+  <si>
+    <t>Sipdus</t>
+  </si>
+  <si>
+    <t>Garantía de obra</t>
+  </si>
+  <si>
+    <t>Said Vargas fortalece estructuras sindicales del SNTE en la Otomí-Tepehua</t>
+  </si>
+  <si>
+    <t>Menchaca no descarta comparecencia del Oficial Mayor ante el Congreso</t>
+  </si>
+  <si>
+    <t>Policía de Ajacuba fortalece acciones de prevención del delito con jornadas sobre prevención del suicidio</t>
+  </si>
+  <si>
+    <t>Policía municipal</t>
+  </si>
+  <si>
+    <t>Prevención del suicidio</t>
+  </si>
+  <si>
+    <t>Pachuca recibirá 1.6 mdp por espacios para Feria</t>
+  </si>
+  <si>
+    <t>Hidalgo será sede de la Olimpiada Nacional 2027; lo oficializa Conade</t>
+  </si>
+  <si>
+    <t>Tuzos enfrentarán a la Selección Mexicana sub 23 en Hidalgo</t>
+  </si>
+  <si>
+    <t>llaa</t>
+  </si>
+  <si>
+    <t>Julio Menchaca respalda labor de universidades tecnológicas y politécnicas</t>
+  </si>
+  <si>
+    <t>Brinda DIFH Hidalgo becas para apoyar la economía familiar de usuarios</t>
+  </si>
+  <si>
+    <t>Tuzas se quedan sin DT: cesan a Óscar Torres</t>
+  </si>
+  <si>
+    <t>¡Late con orgullo!</t>
+  </si>
+  <si>
+    <t>Rodolfo, el niño que se convirtió en El Santo</t>
+  </si>
+  <si>
+    <t>Aniversario natalicio</t>
+  </si>
+  <si>
+    <t>El país supera los 130 millones de habitantes</t>
+  </si>
+  <si>
+    <t>Resultados del ICE 2026 muestran áreas de oportunidad: JMS</t>
+  </si>
+  <si>
+    <t>Seis puertos mexicanos están restringidos por el huracán Polo</t>
+  </si>
+  <si>
+    <t>Alerta Meteorológica</t>
+  </si>
+  <si>
+    <t>Honor a quien honor merece. El personaje de El Santo es sin duda uno de los más queridos en México y sin duda dejó escuela en la lucha libre en nuestro país y en el mundo. Este día conmemoramos con orgullo 109 años de su nacimiento en Tulancingo.</t>
   </si>
 </sst>
 </file>
@@ -838,8 +826,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J61" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J61" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J59" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J59" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J2">
     <sortCondition ref="C1:C2"/>
   </sortState>
@@ -1208,7 +1196,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1257,7 +1245,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B2" t="s">
         <v>67</v>
@@ -1266,32 +1254,32 @@
         <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
         <v>94</v>
       </c>
       <c r="H2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B3" t="s">
         <v>67</v>
@@ -1303,63 +1291,63 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>96</v>
       </c>
       <c r="G3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B4" t="s">
         <v>67</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B5" t="s">
         <v>67</v>
@@ -1368,137 +1356,137 @@
         <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>100</v>
       </c>
       <c r="G5" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="H5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B6" t="s">
         <v>67</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J6" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
-        <v>101</v>
-      </c>
-      <c r="G6" t="s">
-        <v>102</v>
-      </c>
-      <c r="H6" t="s">
-        <v>70</v>
-      </c>
-      <c r="I6" t="str">
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>94</v>
+      </c>
+      <c r="H7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Presidencia de la República</v>
       </c>
-      <c r="J6" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" t="s">
-        <v>98</v>
-      </c>
-      <c r="H7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>106</v>
@@ -1507,50 +1495,50 @@
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -1563,149 +1551,149 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F11" t="s">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="G11" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" t="s">
+        <v>115</v>
+      </c>
+      <c r="G13" t="s">
+        <v>116</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J13" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" t="s">
+        <v>118</v>
+      </c>
+      <c r="H14" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" t="s">
-        <v>72</v>
-      </c>
-      <c r="H13" t="s">
-        <v>11</v>
-      </c>
-      <c r="I13" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J13" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B14" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" t="s">
-        <v>26</v>
-      </c>
-      <c r="F14" t="s">
-        <v>114</v>
-      </c>
-      <c r="G14" t="s">
-        <v>89</v>
-      </c>
-      <c r="H14" t="s">
-        <v>11</v>
-      </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D15" t="s">
         <v>13</v>
@@ -1714,13 +1702,13 @@
         <v>27</v>
       </c>
       <c r="F15" t="s">
-        <v>116</v>
+        <v>27</v>
       </c>
       <c r="G15" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="H15" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -1731,287 +1719,287 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>118</v>
+        <v>71</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D17" t="s">
         <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="F17" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G17" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J17" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" t="s">
+        <v>123</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J17" t="str">
+      <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B18" t="s">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" t="s">
+        <v>89</v>
+      </c>
+      <c r="H19" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D18" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" t="s">
-        <v>45</v>
-      </c>
-      <c r="F18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" t="s">
-        <v>121</v>
-      </c>
-      <c r="H18" t="s">
-        <v>11</v>
-      </c>
-      <c r="I18" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J18" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B19" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="D19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" t="s">
-        <v>123</v>
-      </c>
-      <c r="H19" t="s">
-        <v>11</v>
-      </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F20" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J20" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" t="s">
+        <v>24</v>
+      </c>
+      <c r="G21" t="s">
+        <v>113</v>
+      </c>
+      <c r="H21" t="s">
+        <v>11</v>
+      </c>
+      <c r="I21" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J20" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B21" t="s">
-        <v>78</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" t="s">
-        <v>126</v>
-      </c>
-      <c r="H21" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>127</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E22" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" t="s">
+        <v>128</v>
+      </c>
+      <c r="H22" t="s">
+        <v>11</v>
+      </c>
+      <c r="I22" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J22" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B23" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
         <v>10</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F23" t="s">
         <v>10</v>
       </c>
-      <c r="G22" t="s">
-        <v>126</v>
-      </c>
-      <c r="H22" t="s">
-        <v>11</v>
-      </c>
-      <c r="I22" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J22" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B23" t="s">
-        <v>78</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" t="s">
-        <v>17</v>
-      </c>
       <c r="G23" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="H23" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
@@ -2023,10 +2011,10 @@
         <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="H24" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2039,66 +2027,66 @@
     </row>
     <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
@@ -2107,62 +2095,62 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>84</v>
+        <v>134</v>
       </c>
       <c r="H27" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F28" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G28" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
       <c r="H28" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2170,105 +2158,105 @@
       </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D29" t="s">
-        <v>135</v>
+        <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J29" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" t="s">
+        <v>24</v>
+      </c>
+      <c r="G30" t="s">
+        <v>139</v>
+      </c>
+      <c r="H30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B30" t="s">
-        <v>68</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" t="s">
-        <v>10</v>
-      </c>
-      <c r="F30" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" t="s">
-        <v>137</v>
-      </c>
-      <c r="H30" t="s">
-        <v>70</v>
-      </c>
-      <c r="I30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B31" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F31" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="G31" t="s">
-        <v>139</v>
+        <v>103</v>
       </c>
       <c r="H31" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
@@ -2277,22 +2265,22 @@
     </row>
     <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F32" t="s">
-        <v>27</v>
+        <v>83</v>
       </c>
       <c r="G32" t="s">
         <v>84</v>
@@ -2311,263 +2299,263 @@
     </row>
     <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>143</v>
+      </c>
+      <c r="H33" t="s">
+        <v>69</v>
+      </c>
+      <c r="I33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B34" t="s">
+        <v>74</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>24</v>
+      </c>
+      <c r="F34" t="s">
+        <v>24</v>
+      </c>
+      <c r="G34" t="s">
+        <v>145</v>
+      </c>
+      <c r="H34" t="s">
+        <v>11</v>
+      </c>
+      <c r="I34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>36</v>
+      </c>
+      <c r="F35" t="s">
+        <v>36</v>
+      </c>
+      <c r="G35" t="s">
+        <v>123</v>
+      </c>
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B36" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D36" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" t="s">
+        <v>24</v>
+      </c>
+      <c r="G36" t="s">
+        <v>148</v>
+      </c>
+      <c r="H36" t="s">
+        <v>73</v>
+      </c>
+      <c r="I36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B37" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
         <v>26</v>
       </c>
-      <c r="F33" t="s">
-        <v>2</v>
-      </c>
-      <c r="G33" t="s">
-        <v>98</v>
-      </c>
-      <c r="H33" t="s">
-        <v>11</v>
-      </c>
-      <c r="I33" t="str">
+      <c r="F37" t="s">
+        <v>115</v>
+      </c>
+      <c r="G37" t="s">
+        <v>136</v>
+      </c>
+      <c r="H37" t="s">
+        <v>73</v>
+      </c>
+      <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J33" t="str">
+      <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B34" t="s">
-        <v>76</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D34" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" t="s">
-        <v>17</v>
-      </c>
-      <c r="F34" t="s">
-        <v>17</v>
-      </c>
-      <c r="G34" t="s">
-        <v>143</v>
-      </c>
-      <c r="H34" t="s">
-        <v>11</v>
-      </c>
-      <c r="I34" t="str">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B38" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" t="s">
+        <v>94</v>
+      </c>
+      <c r="H38" t="s">
+        <v>11</v>
+      </c>
+      <c r="I38" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J38" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B39" t="s">
+        <v>74</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>24</v>
+      </c>
+      <c r="F39" t="s">
+        <v>24</v>
+      </c>
+      <c r="G39" t="s">
+        <v>89</v>
+      </c>
+      <c r="H39" t="s">
+        <v>11</v>
+      </c>
+      <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B35" t="s">
-        <v>76</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" t="s">
-        <v>17</v>
-      </c>
-      <c r="F35" t="s">
-        <v>17</v>
-      </c>
-      <c r="G35" t="s">
-        <v>83</v>
-      </c>
-      <c r="H35" t="s">
-        <v>11</v>
-      </c>
-      <c r="I35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A36" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B36" t="s">
-        <v>76</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="D36" t="s">
-        <v>12</v>
-      </c>
-      <c r="E36" t="s">
-        <v>19</v>
-      </c>
-      <c r="F36" t="s">
-        <v>19</v>
-      </c>
-      <c r="G36" t="s">
-        <v>87</v>
-      </c>
-      <c r="H36" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B37" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D37" t="s">
-        <v>9</v>
-      </c>
-      <c r="E37" t="s">
-        <v>27</v>
-      </c>
-      <c r="F37" t="s">
-        <v>2</v>
-      </c>
-      <c r="G37" t="s">
-        <v>84</v>
-      </c>
-      <c r="H37" t="s">
-        <v>11</v>
-      </c>
-      <c r="I37" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J37" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B38" t="s">
-        <v>75</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D38" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" t="s">
-        <v>54</v>
-      </c>
-      <c r="F38" t="s">
-        <v>54</v>
-      </c>
-      <c r="G38" t="s">
-        <v>148</v>
-      </c>
-      <c r="H38" t="s">
-        <v>74</v>
-      </c>
-      <c r="I38" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J38" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B39" t="s">
-        <v>75</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D39" t="s">
-        <v>12</v>
-      </c>
-      <c r="E39" t="s">
-        <v>22</v>
-      </c>
-      <c r="F39" t="s">
-        <v>22</v>
-      </c>
-      <c r="G39" t="s">
-        <v>150</v>
-      </c>
-      <c r="H39" t="s">
-        <v>11</v>
-      </c>
-      <c r="I39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D40" t="s">
-        <v>12</v>
+        <v>153</v>
       </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F40" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G40" t="s">
-        <v>143</v>
+        <v>82</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
@@ -2581,30 +2569,30 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D41" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="E41" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F41" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G41" t="s">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2615,64 +2603,64 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F42" t="s">
-        <v>154</v>
+        <v>78</v>
       </c>
       <c r="G42" t="s">
-        <v>87</v>
+        <v>157</v>
       </c>
       <c r="H42" t="s">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D43" t="s">
-        <v>88</v>
+        <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>26</v>
+        <v>159</v>
       </c>
       <c r="F43" t="s">
-        <v>26</v>
+        <v>159</v>
       </c>
       <c r="G43" t="s">
-        <v>98</v>
+        <v>160</v>
       </c>
       <c r="H43" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2685,50 +2673,50 @@
     </row>
     <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B44" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="G44" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="H44" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B45" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E45" t="s">
         <v>24</v>
@@ -2737,7 +2725,7 @@
         <v>24</v>
       </c>
       <c r="G45" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
@@ -2753,13 +2741,13 @@
     </row>
     <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B46" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
@@ -2768,10 +2756,10 @@
         <v>16</v>
       </c>
       <c r="F46" t="s">
-        <v>79</v>
+        <v>164</v>
       </c>
       <c r="G46" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2785,15 +2773,15 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B47" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
@@ -2805,7 +2793,7 @@
         <v>16</v>
       </c>
       <c r="G47" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
@@ -2821,476 +2809,408 @@
     </row>
     <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B48" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D48" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E48" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F48" t="s">
-        <v>10</v>
+        <v>88</v>
       </c>
       <c r="G48" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="H48" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B49" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>169</v>
       </c>
       <c r="E49" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="G49" t="s">
-        <v>166</v>
+        <v>71</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B50" t="s">
+        <v>81</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>24</v>
+      </c>
+      <c r="F50" t="s">
+        <v>24</v>
+      </c>
+      <c r="G50" t="s">
+        <v>136</v>
+      </c>
+      <c r="H50" t="s">
+        <v>73</v>
+      </c>
+      <c r="I50" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B50" t="s">
-        <v>77</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D50" t="s">
-        <v>80</v>
-      </c>
-      <c r="E50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F50" t="s">
-        <v>10</v>
-      </c>
-      <c r="G50" t="s">
-        <v>168</v>
-      </c>
-      <c r="H50" t="s">
-        <v>11</v>
-      </c>
-      <c r="I50" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B51" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>36</v>
+      </c>
+      <c r="F51" t="s">
+        <v>36</v>
+      </c>
+      <c r="G51" t="s">
+        <v>123</v>
+      </c>
+      <c r="H51" t="s">
+        <v>11</v>
+      </c>
+      <c r="I51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B52" t="s">
+        <v>81</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" t="s">
+        <v>10</v>
+      </c>
+      <c r="G52" t="s">
+        <v>71</v>
+      </c>
+      <c r="H52" t="s">
+        <v>11</v>
+      </c>
+      <c r="I52" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J52" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B53" t="s">
+        <v>81</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D53" t="s">
+        <v>79</v>
+      </c>
+      <c r="E53" t="s">
+        <v>29</v>
+      </c>
+      <c r="F53" t="s">
+        <v>83</v>
+      </c>
+      <c r="G53" t="s">
+        <v>84</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B54" t="s">
+        <v>81</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D54" t="s">
+        <v>79</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" t="s">
+        <v>16</v>
+      </c>
+      <c r="G54" t="s">
+        <v>92</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B55" t="s">
+        <v>86</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D55" t="s">
         <v>13</v>
       </c>
-      <c r="E51" t="s">
-        <v>27</v>
-      </c>
-      <c r="F51" t="s">
-        <v>2</v>
-      </c>
-      <c r="G51" t="s">
-        <v>84</v>
-      </c>
-      <c r="H51" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J51" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A52" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B52" t="s">
-        <v>82</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D52" t="s">
-        <v>12</v>
-      </c>
-      <c r="E52" t="s">
-        <v>29</v>
-      </c>
-      <c r="F52" t="s">
-        <v>86</v>
-      </c>
-      <c r="G52" t="s">
-        <v>87</v>
-      </c>
-      <c r="H52" t="s">
-        <v>11</v>
-      </c>
-      <c r="I52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A53" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B53" t="s">
-        <v>82</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D53" t="s">
-        <v>12</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="E55" t="s">
         <v>10</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F55" t="s">
         <v>10</v>
       </c>
-      <c r="G53" t="s">
-        <v>172</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A54" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B54" t="s">
-        <v>82</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="D54" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" t="s">
-        <v>26</v>
-      </c>
-      <c r="F54" t="s">
-        <v>2</v>
-      </c>
-      <c r="G54" t="s">
-        <v>174</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B55" t="s">
-        <v>82</v>
-      </c>
-      <c r="C55" s="5" t="s">
+      <c r="G55" t="s">
         <v>175</v>
       </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>24</v>
-      </c>
-      <c r="F55" t="s">
-        <v>24</v>
-      </c>
-      <c r="G55" t="s">
-        <v>158</v>
-      </c>
       <c r="H55" t="s">
         <v>11</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gobernador</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="11">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B56" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>176</v>
       </c>
       <c r="D56" t="s">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F56" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G56" t="s">
+        <v>94</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B57" t="s">
+        <v>86</v>
+      </c>
+      <c r="C57" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F57" t="s">
+        <v>24</v>
+      </c>
+      <c r="G57" t="s">
+        <v>89</v>
+      </c>
+      <c r="H57" t="s">
+        <v>11</v>
+      </c>
+      <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B57" t="s">
-        <v>82</v>
-      </c>
-      <c r="C57" s="5" t="s">
+      <c r="J57" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B58" t="s">
+        <v>86</v>
+      </c>
+      <c r="C58" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="D57" t="s">
-        <v>80</v>
-      </c>
-      <c r="E57" t="s">
-        <v>16</v>
-      </c>
-      <c r="F57" t="s">
-        <v>16</v>
-      </c>
-      <c r="G57" t="s">
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58" t="s">
         <v>179</v>
       </c>
-      <c r="H57" t="s">
-        <v>11</v>
-      </c>
-      <c r="I57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B58" t="s">
-        <v>90</v>
-      </c>
-      <c r="C58" s="5" t="s">
+      <c r="H58" t="s">
+        <v>11</v>
+      </c>
+      <c r="I58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A59" s="11">
+        <v>46288</v>
+      </c>
+      <c r="B59" t="s">
+        <v>86</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="D58" t="s">
-        <v>13</v>
-      </c>
-      <c r="E58" t="s">
-        <v>27</v>
-      </c>
-      <c r="F58" t="s">
-        <v>27</v>
-      </c>
-      <c r="G58" t="s">
-        <v>84</v>
-      </c>
-      <c r="H58" t="s">
-        <v>70</v>
-      </c>
-      <c r="I58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B59" t="s">
-        <v>90</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>181</v>
-      </c>
       <c r="D59" t="s">
-        <v>12</v>
+        <v>153</v>
       </c>
       <c r="E59" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F59" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G59" t="s">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="H59" t="s">
         <v>11</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B60" t="s">
-        <v>90</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D60" t="s">
-        <v>12</v>
-      </c>
-      <c r="E60" t="s">
-        <v>26</v>
-      </c>
-      <c r="F60" t="s">
-        <v>26</v>
-      </c>
-      <c r="G60" t="s">
-        <v>98</v>
-      </c>
-      <c r="H60" t="s">
-        <v>11</v>
-      </c>
-      <c r="I60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="11">
-        <v>46287</v>
-      </c>
-      <c r="B61" t="s">
-        <v>90</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="D61" t="s">
-        <v>12</v>
-      </c>
-      <c r="E61" t="s">
-        <v>58</v>
-      </c>
-      <c r="F61" t="s">
-        <v>58</v>
-      </c>
-      <c r="G61" t="s">
-        <v>184</v>
-      </c>
-      <c r="H61" t="s">
-        <v>11</v>
-      </c>
-      <c r="I61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Otros</v>
       </c>
@@ -3350,7 +3270,7 @@
         <v>31</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
         <v>66</v>
@@ -3386,7 +3306,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
         <v>32</v>
@@ -3862,7 +3782,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B49" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
Corregido Presupuesto de Egresos
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Repositorios de capturas y reportes\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28E6AF2-B958-4781-8103-5D1ECF0D17F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4B3B42-823E-4A6D-8B16-9AFECE3F3D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -394,9 +394,6 @@
     <t>Estiman ingresos por 79 mil mdp</t>
   </si>
   <si>
-    <t>Ley De Ingresos</t>
-  </si>
-  <si>
     <t>Analizan Hoy No Circula para Pachuca</t>
   </si>
   <si>
@@ -635,6 +632,9 @@
   </si>
   <si>
     <t>Prevención De Enfermedades</t>
+  </si>
+  <si>
+    <t>Presupuesto de egresos</t>
   </si>
 </sst>
 </file>
@@ -793,14 +793,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill>
@@ -1929,12 +1922,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J71" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J71" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5">
   <autoFilter ref="A1:J71" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
-    <tableColumn id="3" xr3:uid="{4CA37DD5-010E-43EE-907D-87C1845DB2AB}" name="Titular" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{4CA37DD5-010E-43EE-907D-87C1845DB2AB}" name="Titular" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{1E763E28-25D7-4FE7-AD1A-91C7A0FE0E7A}" name="Recurso editorial"/>
     <tableColumn id="5" xr3:uid="{F8C19AF2-6D19-449B-9F8B-6424964B1BCF}" name="Dependencia"/>
     <tableColumn id="6" xr3:uid="{46DF0510-7A9A-4625-979E-4EBC30CC7AA3}" name="Organismo"/>
@@ -1966,13 +1959,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80AFAA35-C663-4971-9820-992B55167F9C}" name="Tabla3" displayName="Tabla3" ref="D1:E27" totalsRowShown="0" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80AFAA35-C663-4971-9820-992B55167F9C}" name="Tabla3" displayName="Tabla3" ref="D1:E27" totalsRowShown="0" tableBorderDxfId="2">
   <autoFilter ref="D1:E27" xr:uid="{80AFAA35-C663-4971-9820-992B55167F9C}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D2:E27">
     <sortCondition ref="D1:D27"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A040A308-8C62-4D4B-B3BE-EC124A9B961C}" name="Dependencia" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{A040A308-8C62-4D4B-B3BE-EC124A9B961C}" name="Dependencia" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{2B2FFCF1-496A-4D37-8C8B-790A66FD9968}" name="Nivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2985,7 +2978,7 @@
         <v>2</v>
       </c>
       <c r="G10" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
@@ -3007,7 +3000,7 @@
         <v>69</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
@@ -3019,7 +3012,7 @@
         <v>27</v>
       </c>
       <c r="G11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
@@ -3041,7 +3034,7 @@
         <v>69</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -3053,7 +3046,7 @@
         <v>17</v>
       </c>
       <c r="G12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
@@ -3075,7 +3068,7 @@
         <v>69</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D13" t="s">
         <v>9</v>
@@ -3087,7 +3080,7 @@
         <v>24</v>
       </c>
       <c r="G13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -3109,7 +3102,7 @@
         <v>71</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -3143,7 +3136,7 @@
         <v>71</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -3177,7 +3170,7 @@
         <v>71</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D16" t="s">
         <v>13</v>
@@ -3189,7 +3182,7 @@
         <v>27</v>
       </c>
       <c r="G16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
@@ -3211,7 +3204,7 @@
         <v>71</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -3223,7 +3216,7 @@
         <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -3245,7 +3238,7 @@
         <v>71</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
@@ -3254,7 +3247,7 @@
         <v>61</v>
       </c>
       <c r="F18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G18" t="s">
         <v>61</v>
@@ -3279,7 +3272,7 @@
         <v>71</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
@@ -3313,7 +3306,7 @@
         <v>71</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
@@ -3325,7 +3318,7 @@
         <v>24</v>
       </c>
       <c r="G20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
@@ -3347,7 +3340,7 @@
         <v>74</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D21" t="s">
         <v>13</v>
@@ -3381,7 +3374,7 @@
         <v>74</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
@@ -3393,7 +3386,7 @@
         <v>39</v>
       </c>
       <c r="G22" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
@@ -3415,7 +3408,7 @@
         <v>74</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
@@ -3449,7 +3442,7 @@
         <v>74</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
@@ -3483,7 +3476,7 @@
         <v>74</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D25" t="s">
         <v>9</v>
@@ -3495,7 +3488,7 @@
         <v>24</v>
       </c>
       <c r="G25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H25" t="s">
         <v>72</v>
@@ -3517,7 +3510,7 @@
         <v>74</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
@@ -3529,7 +3522,7 @@
         <v>26</v>
       </c>
       <c r="G26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
@@ -3551,7 +3544,7 @@
         <v>74</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -3563,7 +3556,7 @@
         <v>16</v>
       </c>
       <c r="G27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
@@ -3585,7 +3578,7 @@
         <v>74</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
@@ -3597,7 +3590,7 @@
         <v>18</v>
       </c>
       <c r="G28" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
@@ -3619,7 +3612,7 @@
         <v>74</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
@@ -3653,7 +3646,7 @@
         <v>74</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
@@ -3687,7 +3680,7 @@
         <v>74</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
@@ -3721,7 +3714,7 @@
         <v>77</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
@@ -3755,7 +3748,7 @@
         <v>77</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
@@ -3767,7 +3760,7 @@
         <v>39</v>
       </c>
       <c r="G33" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
@@ -3789,7 +3782,7 @@
         <v>77</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
@@ -3823,7 +3816,7 @@
         <v>77</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
@@ -3857,7 +3850,7 @@
         <v>77</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
@@ -3866,7 +3859,7 @@
         <v>61</v>
       </c>
       <c r="F36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G36" t="s">
         <v>90</v>
@@ -3891,7 +3884,7 @@
         <v>73</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D37" t="s">
         <v>13</v>
@@ -3903,7 +3896,7 @@
         <v>2</v>
       </c>
       <c r="G37" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
@@ -3925,7 +3918,7 @@
         <v>73</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
@@ -3937,7 +3930,7 @@
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -3959,7 +3952,7 @@
         <v>73</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
@@ -3993,7 +3986,7 @@
         <v>73</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
@@ -4027,7 +4020,7 @@
         <v>73</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
@@ -4061,7 +4054,7 @@
         <v>76</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D42" t="s">
         <v>13</v>
@@ -4073,7 +4066,7 @@
         <v>39</v>
       </c>
       <c r="G42" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
@@ -4095,7 +4088,7 @@
         <v>76</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
@@ -4107,7 +4100,7 @@
         <v>24</v>
       </c>
       <c r="G43" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
@@ -4129,7 +4122,7 @@
         <v>76</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
@@ -4163,7 +4156,7 @@
         <v>76</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
@@ -4197,7 +4190,7 @@
         <v>88</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D46" t="s">
         <v>13</v>
@@ -4231,7 +4224,7 @@
         <v>88</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
@@ -4243,7 +4236,7 @@
         <v>2</v>
       </c>
       <c r="G47" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
@@ -4265,7 +4258,7 @@
         <v>88</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D48" t="s">
         <v>9</v>
@@ -4277,7 +4270,7 @@
         <v>24</v>
       </c>
       <c r="G48" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
@@ -4299,7 +4292,7 @@
         <v>88</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
@@ -4311,7 +4304,7 @@
         <v>24</v>
       </c>
       <c r="G49" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
@@ -4333,7 +4326,7 @@
         <v>88</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -4345,7 +4338,7 @@
         <v>27</v>
       </c>
       <c r="G50" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
@@ -4367,7 +4360,7 @@
         <v>88</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
@@ -4379,7 +4372,7 @@
         <v>39</v>
       </c>
       <c r="G51" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -4401,7 +4394,7 @@
         <v>80</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
         <v>81</v>
@@ -4435,7 +4428,7 @@
         <v>80</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D53" t="s">
         <v>12</v>
@@ -4503,7 +4496,7 @@
         <v>80</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D55" t="s">
         <v>9</v>
@@ -4515,7 +4508,7 @@
         <v>24</v>
       </c>
       <c r="G55" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H55" t="s">
         <v>72</v>
@@ -4537,7 +4530,7 @@
         <v>80</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
@@ -4549,7 +4542,7 @@
         <v>92</v>
       </c>
       <c r="G56" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
@@ -4571,7 +4564,7 @@
         <v>80</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
@@ -4583,7 +4576,7 @@
         <v>25</v>
       </c>
       <c r="G57" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
@@ -4605,7 +4598,7 @@
         <v>80</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -4617,7 +4610,7 @@
         <v>83</v>
       </c>
       <c r="G58" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
@@ -4639,7 +4632,7 @@
         <v>80</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D59" t="s">
         <v>12</v>
@@ -4673,7 +4666,7 @@
         <v>80</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D60" t="s">
         <v>12</v>
@@ -4685,7 +4678,7 @@
         <v>10</v>
       </c>
       <c r="G60" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
@@ -4707,7 +4700,7 @@
         <v>80</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
@@ -4719,7 +4712,7 @@
         <v>24</v>
       </c>
       <c r="G61" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
@@ -4741,7 +4734,7 @@
         <v>80</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D62" t="s">
         <v>12</v>
@@ -4753,7 +4746,7 @@
         <v>16</v>
       </c>
       <c r="G62" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
@@ -4775,7 +4768,7 @@
         <v>80</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
@@ -4787,7 +4780,7 @@
         <v>16</v>
       </c>
       <c r="G63" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
@@ -4809,7 +4802,7 @@
         <v>80</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D64" t="s">
         <v>78</v>
@@ -4843,7 +4836,7 @@
         <v>89</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D65" t="s">
         <v>13</v>
@@ -4877,7 +4870,7 @@
         <v>89</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D66" t="s">
         <v>12</v>
@@ -4889,7 +4882,7 @@
         <v>24</v>
       </c>
       <c r="G66" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H66" t="s">
         <v>72</v>
@@ -4911,7 +4904,7 @@
         <v>89</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D67" t="s">
         <v>12</v>
@@ -4923,7 +4916,7 @@
         <v>2</v>
       </c>
       <c r="G67" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="H67" t="s">
         <v>11</v>
@@ -4945,7 +4938,7 @@
         <v>89</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D68" t="s">
         <v>12</v>
@@ -4979,7 +4972,7 @@
         <v>89</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D69" t="s">
         <v>12</v>
@@ -4991,7 +4984,7 @@
         <v>2</v>
       </c>
       <c r="G69" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H69" t="s">
         <v>11</v>
@@ -5013,7 +5006,7 @@
         <v>89</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D70" t="s">
         <v>78</v>
@@ -5025,7 +5018,7 @@
         <v>15</v>
       </c>
       <c r="G70" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H70" t="s">
         <v>11</v>
@@ -5075,7 +5068,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I71">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$I2="XXX"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>